<commit_message>
Create script to generate regional extracts and generate extract for CEDS region
</commit_message>
<xml_diff>
--- a/deliverables/regional_extracts/County Controls - CEDS Region.xlsx
+++ b/deliverables/regional_extracts/County Controls - CEDS Region.xlsx
@@ -1,22 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://morpc1-my.sharepoint.com/personal/aporr_morpc_org/Documents/morpc-county-controls/deliverables/regional_extracts/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_1EBE8CB8CAEBC80A22F575085782CCAA7A398263" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Total population" sheetId="1" r:id="rId1"/>
-    <sheet name="Population change" sheetId="2" r:id="rId2"/>
-    <sheet name="Jobs change" sheetId="3" r:id="rId3"/>
+    <sheet name="Detailed population forecast" sheetId="1" r:id="rId1"/>
+    <sheet name="Population" sheetId="2" r:id="rId2"/>
+    <sheet name="Households" sheetId="3" r:id="rId3"/>
+    <sheet name="Housing units" sheetId="4" r:id="rId4"/>
+    <sheet name="Jobs" sheetId="5" r:id="rId5"/>
+    <sheet name="Population by age" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="118">
   <si>
     <t>Forecasted population</t>
   </si>
@@ -149,6 +158,142 @@
 (+32%)</t>
   </si>
   <si>
+    <t>Households</t>
+  </si>
+  <si>
+    <t>Households label</t>
+  </si>
+  <si>
+    <t>862,800</t>
+  </si>
+  <si>
+    <t>866,200</t>
+  </si>
+  <si>
+    <t>912,700</t>
+  </si>
+  <si>
+    <t>958,100</t>
+  </si>
+  <si>
+    <t>1,014,300</t>
+  </si>
+  <si>
+    <t>1,058,200</t>
+  </si>
+  <si>
+    <t>1,095,800</t>
+  </si>
+  <si>
+    <t>1,133,500</t>
+  </si>
+  <si>
+    <t>+27%</t>
+  </si>
+  <si>
+    <t>+31%</t>
+  </si>
+  <si>
+    <t>862,800
+(+0%)</t>
+  </si>
+  <si>
+    <t>866,200
+(+0%)</t>
+  </si>
+  <si>
+    <t>912,700
+(+6%)</t>
+  </si>
+  <si>
+    <t>958,100
+(+11%)</t>
+  </si>
+  <si>
+    <t>1,014,300
+(+18%)</t>
+  </si>
+  <si>
+    <t>1,058,200
+(+23%)</t>
+  </si>
+  <si>
+    <t>1,095,800
+(+27%)</t>
+  </si>
+  <si>
+    <t>1,133,500
+(+31%)</t>
+  </si>
+  <si>
+    <t>Housing units</t>
+  </si>
+  <si>
+    <t>Housing units label</t>
+  </si>
+  <si>
+    <t>934,700</t>
+  </si>
+  <si>
+    <t>938,200</t>
+  </si>
+  <si>
+    <t>988,200</t>
+  </si>
+  <si>
+    <t>1,036,900</t>
+  </si>
+  <si>
+    <t>1,097,300</t>
+  </si>
+  <si>
+    <t>1,144,300</t>
+  </si>
+  <si>
+    <t>1,184,600</t>
+  </si>
+  <si>
+    <t>1,224,900</t>
+  </si>
+  <si>
+    <t>+17%</t>
+  </si>
+  <si>
+    <t>+22%</t>
+  </si>
+  <si>
+    <t>934,700
+(+0%)</t>
+  </si>
+  <si>
+    <t>938,200
+(+0%)</t>
+  </si>
+  <si>
+    <t>988,200
+(+6%)</t>
+  </si>
+  <si>
+    <t>1,036,900
+(+11%)</t>
+  </si>
+  <si>
+    <t>1,097,300
+(+17%)</t>
+  </si>
+  <si>
+    <t>1,144,300
+(+22%)</t>
+  </si>
+  <si>
+    <t>1,184,600
+(+27%)</t>
+  </si>
+  <si>
+    <t>1,224,900
+(+31%)</t>
+  </si>
+  <si>
     <t>Total jobs</t>
   </si>
   <si>
@@ -248,18 +393,31 @@
   <si>
     <t>1,563,600
 (+30%)</t>
+  </si>
+  <si>
+    <t>Population ages 17 and under</t>
+  </si>
+  <si>
+    <t>Population ages 18 to 64</t>
+  </si>
+  <si>
+    <t>Population ages 65 and older</t>
+  </si>
+  <si>
+    <t>Population ages 17 and under (percent)</t>
+  </si>
+  <si>
+    <t>Population ages 18 to 64 (percent)</t>
+  </si>
+  <si>
+    <t>Population ages 65 and older (percent)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="@"/>
-  </numFmts>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,24 +471,42 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -352,18 +528,20 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
+      <c:overlay val="0"/>
     </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Total population'!$B$1</c:f>
+              <c:f>'Detailed population forecast'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -392,10 +570,9 @@
             </c:spPr>
           </c:marker>
           <c:cat>
-            <c:numRef>
-              <c:f>'Total population'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>'Detailed population forecast'!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -421,14 +598,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Total population'!$B$2:$B$9</c:f>
+              <c:f>'Detailed population forecast'!$B$2:$B$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2251797</c:v>
@@ -457,13 +634,19 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FA55-447E-B907-785176378AC3}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Total population'!$C$1</c:f>
+              <c:f>'Detailed population forecast'!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -492,10 +675,9 @@
             </c:spPr>
           </c:marker>
           <c:cat>
-            <c:numRef>
-              <c:f>'Total population'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>'Detailed population forecast'!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -521,14 +703,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Total population'!$C$2:$C$9</c:f>
+              <c:f>'Detailed population forecast'!$C$2:$C$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="2">
                   <c:v>2281046</c:v>
@@ -551,13 +733,19 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FA55-447E-B907-785176378AC3}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Total population'!$D$1</c:f>
+              <c:f>'Detailed population forecast'!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -586,10 +774,9 @@
             </c:spPr>
           </c:marker>
           <c:cat>
-            <c:numRef>
-              <c:f>'Total population'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>'Detailed population forecast'!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -615,14 +802,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Total population'!$D$2:$D$9</c:f>
+              <c:f>'Detailed population forecast'!$D$2:$D$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="2">
                   <c:v>2420418</c:v>
@@ -645,8 +832,23 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-FA55-447E-B907-785176378AC3}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:marker val="1"/>
+        <c:smooth val="0"/>
         <c:axId val="50010001"/>
         <c:axId val="50010002"/>
       </c:lineChart>
@@ -655,8 +857,11 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -675,15 +880,19 @@
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="50010002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -704,7 +913,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
+      <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
@@ -719,6 +928,8 @@
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -729,8 +940,18 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -752,19 +973,21 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
+      <c:overlay val="0"/>
     </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Population change'!$B$1</c:f>
+              <c:f>Population!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -781,11 +1004,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Population change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Population!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -811,14 +1034,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Population change'!$B$2:$B$9</c:f>
+              <c:f>Population!$B$2:$B$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2251797</c:v>
@@ -847,7 +1070,21 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-60D8-4043-B466-59406681E754}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
         <c:axId val="50020001"/>
         <c:axId val="50020002"/>
       </c:barChart>
@@ -856,8 +1093,11 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -876,15 +1116,19 @@
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="50020002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -904,6 +1148,8 @@
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -914,8 +1160,458 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>CEDS Region forecasted households with percent change since 2020</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Households!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Households</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2C7F68"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Households!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Households!$B$2:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>862783</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>866170</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>912706</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>958107</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1014325</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1058178</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1095850</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1133524</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3485-45FE-8680-1E51707DE548}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="50030001"/>
+        <c:axId val="50030002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50030001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50030002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50030002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50030001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>CEDS Region forecasted housing units with percent change since 2020</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Housing units'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Housing units</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2C6179"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Housing units'!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Housing units'!$B$2:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>934660</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>938246</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>988218</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1036891</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1097262</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1144257</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1184571</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1224885</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1E43-4479-B066-36946D66C8A8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="50040001"/>
+        <c:axId val="50040002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50040001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50040002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50040002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50040001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -937,19 +1633,21 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
+      <c:overlay val="0"/>
     </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Jobs change'!$D$1</c:f>
+              <c:f>Jobs!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -966,11 +1664,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Jobs change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Jobs!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -996,14 +1694,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Jobs change'!$D$2:$D$9</c:f>
+              <c:f>Jobs!$D$2:$D$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>501639</c:v>
@@ -1032,13 +1730,18 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9F52-453E-BA35-3BC94DC34EC2}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Jobs change'!$E$1</c:f>
+              <c:f>Jobs!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1055,11 +1758,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Jobs change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Jobs!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -1085,14 +1788,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Jobs change'!$E$2:$E$9</c:f>
+              <c:f>Jobs!$E$2:$E$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>112902</c:v>
@@ -1121,13 +1824,18 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9F52-453E-BA35-3BC94DC34EC2}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Jobs change'!$F$1</c:f>
+              <c:f>Jobs!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1144,11 +1852,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Jobs change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Jobs!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -1174,14 +1882,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Jobs change'!$F$2:$F$9</c:f>
+              <c:f>Jobs!$F$2:$F$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>138249</c:v>
@@ -1210,13 +1918,18 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-9F52-453E-BA35-3BC94DC34EC2}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Jobs change'!$C$1</c:f>
+              <c:f>Jobs!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1233,11 +1946,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Jobs change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Jobs!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -1263,14 +1976,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Jobs change'!$C$2:$C$9</c:f>
+              <c:f>Jobs!$C$2:$C$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>255588</c:v>
@@ -1299,13 +2012,18 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-9F52-453E-BA35-3BC94DC34EC2}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Jobs change'!$G$1</c:f>
+              <c:f>Jobs!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1322,11 +2040,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:numRef>
-              <c:f>'Jobs change'!$A$2:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+            <c:strRef>
+              <c:f>Jobs!$A$2:$A$9</c:f>
+              <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2020</c:v>
@@ -1352,14 +2070,14 @@
                 <c:pt idx="7">
                   <c:v>2050</c:v>
                 </c:pt>
-              </c:numCache>
-            </c:numRef>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Jobs change'!$G$2:$G$9</c:f>
+              <c:f>Jobs!$G$2:$G$9</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>197517</c:v>
@@ -1388,18 +2106,35 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-9F52-453E-BA35-3BC94DC34EC2}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="50030001"/>
-        <c:axId val="50030002"/>
+        <c:axId val="50050001"/>
+        <c:axId val="50050002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50030001"/>
+        <c:axId val="50050001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -1413,20 +2148,24 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50030002"/>
+        <c:crossAx val="50050002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50030002"/>
+        <c:axId val="50050002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:txPr>
           <a:bodyPr/>
@@ -1440,14 +2179,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50030001"/>
+        <c:crossAx val="50050001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
+      <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
@@ -1462,6 +2201,433 @@
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>CEDS Region forecasted population by age</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Population by age'!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Population ages 17 and under (percent)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E5072"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Population by age'!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Population by age'!$F$2:$F$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.2333984813018225</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.23373257879198811</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.23112231503529909</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.22912281373950619</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.22672896633030881</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.22588279349517351</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.22412846029493869</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.2230690950963056</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5E9E-450D-AC5A-DC1EA56512EE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Population by age'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Population ages 18 to 64 (percent)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="00B2BF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Population by age'!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Population by age'!$G$2:$G$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.62408822820174292</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.62372401437336711</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.61151772166868945</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.60279006391451884</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.60210440278578181</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.60464387204351078</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.60949681348625628</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.61068405012991189</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5E9E-450D-AC5A-DC1EA56512EE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Population by age'!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Population ages 65 and older (percent)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0077BF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Population by age'!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Population by age'!$H$2:$H$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.1425132904964346</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.14254340683464481</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.15735996329601151</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.16808712234597489</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1711666308839094</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.16947333446131571</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.16637472621880489</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.16624685477378251</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-5E9E-450D-AC5A-DC1EA56512EE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50060001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50060002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50060002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50060001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" baseline="0">
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -1488,7 +2654,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1523,7 +2695,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1545,6 +2723,88 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
@@ -1558,7 +2818,54 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1577,9 +2884,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1617,7 +2924,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1651,6 +2958,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1685,9 +2993,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1860,16 +3169,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="1" customWidth="1"/>
+    <col min="2" max="4" width="12.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -1883,7 +3190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1891,7 +3198,7 @@
         <v>2251797</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1899,7 +3206,7 @@
         <v>2261683</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1913,7 +3220,7 @@
         <v>2420418</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1927,7 +3234,7 @@
         <v>2628330</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1941,7 +3248,7 @@
         <v>2865039</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1955,7 +3262,7 @@
         <v>3125373</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1969,7 +3276,7 @@
         <v>3406243</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -1990,19 +3297,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" style="4" customWidth="1"/>
+    <col min="2" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" style="3" customWidth="1"/>
+    <col min="5" max="7" width="12.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -2025,7 +3329,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2048,7 +3352,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -2059,7 +3363,7 @@
         <v>9886</v>
       </c>
       <c r="D3" s="3">
-        <v>0.004390271414341524</v>
+        <v>4.390271414341524E-3</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>19</v>
@@ -2071,7 +3375,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -2082,7 +3386,7 @@
         <v>132685</v>
       </c>
       <c r="D4" s="3">
-        <v>0.05892405043616276</v>
+        <v>5.8924050436162757E-2</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>20</v>
@@ -2094,7 +3398,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -2105,7 +3409,7 @@
         <v>253737</v>
       </c>
       <c r="D5" s="3">
-        <v>0.1126820046389617</v>
+        <v>0.11268200463896171</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>21</v>
@@ -2117,7 +3421,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -2140,7 +3444,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -2151,7 +3455,7 @@
         <v>520114</v>
       </c>
       <c r="D7" s="3">
-        <v>0.2309773039043928</v>
+        <v>0.23097730390439281</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>23</v>
@@ -2163,7 +3467,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2174,7 +3478,7 @@
         <v>620935</v>
       </c>
       <c r="D8" s="3">
-        <v>0.2757508780764873</v>
+        <v>0.27575087807648729</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>24</v>
@@ -2186,7 +3490,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -2197,7 +3501,7 @@
         <v>721757</v>
       </c>
       <c r="D9" s="3">
-        <v>0.3205248963383467</v>
+        <v>0.32052489633834669</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>25</v>
@@ -2216,24 +3520,16 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" style="4" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" style="4" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" style="4" customWidth="1"/>
+    <col min="2" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" style="3" customWidth="1"/>
+    <col min="5" max="7" width="12.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -2241,28 +3537,474 @@
         <v>41</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>862783</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1">
+        <v>866170</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3387</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3.9256684473384382E-3</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>912706</v>
+      </c>
+      <c r="C4" s="1">
+        <v>49923</v>
+      </c>
+      <c r="D4" s="3">
+        <v>5.7862753438581889E-2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1">
+        <v>958107</v>
+      </c>
+      <c r="C5" s="1">
+        <v>95324</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.11048432804077039</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1014325</v>
+      </c>
+      <c r="C6" s="1">
+        <v>151542</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.17564323821864819</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1058178</v>
+      </c>
+      <c r="C7" s="1">
+        <v>195395</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.22647061891576439</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1095850</v>
+      </c>
+      <c r="C8" s="1">
+        <v>233067</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.27013397343248541</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1133524</v>
+      </c>
+      <c r="C9" s="1">
+        <v>270741</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.31379964602918692</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" style="3" customWidth="1"/>
+    <col min="5" max="7" width="12.6640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="D1" s="2" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>46</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>934660</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1">
+        <v>938246</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3586</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3.836689277384289E-3</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>988218</v>
+      </c>
+      <c r="C4" s="1">
+        <v>53558</v>
+      </c>
+      <c r="D4" s="3">
+        <v>5.7302120557207972E-2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1036891</v>
+      </c>
+      <c r="C5" s="1">
+        <v>102231</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.1093777416386707</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1097262</v>
+      </c>
+      <c r="C6" s="1">
+        <v>162602</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.17396914385979931</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1144257</v>
+      </c>
+      <c r="C7" s="1">
+        <v>209597</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.22424945969657409</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1184571</v>
+      </c>
+      <c r="C8" s="1">
+        <v>249911</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.26738172169558982</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1224885</v>
+      </c>
+      <c r="C9" s="1">
+        <v>290225</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.31051398369460548</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="8" width="12.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" style="3" customWidth="1"/>
+    <col min="10" max="12" width="12.6640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>16</v>
@@ -2271,7 +4013,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2300,16 +4042,16 @@
         <v>0</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -2335,19 +4077,19 @@
         <v>10910</v>
       </c>
       <c r="I3" s="3">
-        <v>0.00904722218766974</v>
+        <v>9.0472221876697397E-3</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>57</v>
+        <v>97</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -2373,19 +4115,19 @@
         <v>54533</v>
       </c>
       <c r="I4" s="3">
-        <v>0.045222013525224</v>
+        <v>4.5222013525224002E-2</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -2411,19 +4153,19 @@
         <v>100333</v>
       </c>
       <c r="I5" s="3">
-        <v>0.08320210300233437</v>
+        <v>8.3202103002334368E-2</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -2449,19 +4191,19 @@
         <v>179425</v>
       </c>
       <c r="I6" s="3">
-        <v>0.1487899029351643</v>
+        <v>0.14878990293516431</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -2487,19 +4229,19 @@
         <v>244711</v>
       </c>
       <c r="I7" s="3">
-        <v>0.2029289448915536</v>
+        <v>0.20292894489155361</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2525,19 +4267,19 @@
         <v>303517</v>
       </c>
       <c r="I8" s="3">
-        <v>0.2516943846686486</v>
+        <v>0.25169438466864857</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -2563,16 +4305,265 @@
         <v>357716</v>
       </c>
       <c r="I9" s="3">
-        <v>0.2966394254889522</v>
+        <v>0.29663942548895222</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>71</v>
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="5" width="12.6640625" style="1" customWidth="1"/>
+    <col min="6" max="8" width="12.6640625" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2251797</v>
+      </c>
+      <c r="C2" s="1">
+        <v>525566</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1405320</v>
+      </c>
+      <c r="E2" s="1">
+        <v>320911</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0.2333984813018225</v>
+      </c>
+      <c r="G2" s="3">
+        <v>0.62408822820174292</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0.1425132904964346</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2261683</v>
+      </c>
+      <c r="C3" s="1">
+        <v>528629</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1410666</v>
+      </c>
+      <c r="E3" s="1">
+        <v>322388</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.23373257879198811</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0.62372401437336711</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.14254340683464481</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2384482</v>
+      </c>
+      <c r="C4" s="1">
+        <v>551107</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1458153</v>
+      </c>
+      <c r="E4" s="1">
+        <v>375222</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0.23112231503529909</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0.61151772166868945</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.15735996329601151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2505534</v>
+      </c>
+      <c r="C5" s="1">
+        <v>574075</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1510311</v>
+      </c>
+      <c r="E5" s="1">
+        <v>421148</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0.22912281373950619</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0.60279006391451884</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.16808712234597489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2654910</v>
+      </c>
+      <c r="C6" s="1">
+        <v>601945</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1598533</v>
+      </c>
+      <c r="E6" s="1">
+        <v>454432</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0.22672896633030881</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0.60210440278578181</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.1711666308839094</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2771911</v>
+      </c>
+      <c r="C7" s="1">
+        <v>626127</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1676019</v>
+      </c>
+      <c r="E7" s="1">
+        <v>469765</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0.22588279349517351</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0.60464387204351078</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0.16947333446131571</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2872732</v>
+      </c>
+      <c r="C8" s="1">
+        <v>643861</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1750921</v>
+      </c>
+      <c r="E8" s="1">
+        <v>477950</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0.22412846029493869</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0.60949681348625628</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0.16637472621880489</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2973554</v>
+      </c>
+      <c r="C9" s="1">
+        <v>663308</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1815902</v>
+      </c>
+      <c r="E9" s="1">
+        <v>494344</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0.2230690950963056</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0.61068405012991189</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.16624685477378251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>